<commit_message>
feat(ai): clean readme figures step 3 methodology and pure english headers
</commit_message>
<xml_diff>
--- a/data/analyze/post_rescued_nrc_630_codebook.xlsx
+++ b/data/analyze/post_rescued_nrc_630_codebook.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2525" uniqueCount="1386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2525" uniqueCount="1280">
   <si>
     <t>word</t>
   </si>
@@ -25,7 +25,7 @@
     <t>frequency_21215</t>
   </si>
   <si>
-    <t>chinese_translation</t>
+    <t>english_translation</t>
   </si>
   <si>
     <t>category_and_emotion</t>
@@ -3781,397 +3781,79 @@
     <t>刺激快感</t>
   </si>
   <si>
-    <t>1a. 原生 NRC 8大情绪词</t>
-  </si>
-  <si>
-    <t>1b. 原生 NRC 极性词</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (respectful -&gt; respectful)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (immaculate -&gt; immaculate)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (annoying -&gt; annoying)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (fuss -&gt; fuss)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (awful -&gt; awful)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (awed -&gt; awed)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (bubbly -&gt; bubbly)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (praise -&gt; praise)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (trustworthy -&gt; trustworthy)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (satisfaction -&gt; satisfaction)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (ruined -&gt; ruined)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (proud -&gt; proud)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (marvellous -&gt; marvellous)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (intrusive -&gt; intrusive)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (glowing -&gt; glowing)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (frustrating -&gt; frustrating)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (bothered -&gt; bothered)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (authentic -&gt; authentic)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (tricky -&gt; tricky)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (worldly -&gt; worldly)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (vibrant -&gt; vibrant)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (uneasy -&gt; uneasy)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (precious -&gt; precious)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (safest -&gt; safest)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (responsible -&gt; responsible)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (pleasurable -&gt; pleasurable)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (apologetic -&gt; apologetic)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (bored -&gt; bored)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (soaking -&gt; soaking)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (stuffy -&gt; stuffy)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (superbly -&gt; superbly)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (wondrous -&gt; wondrous)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (satisfying -&gt; satisfying)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (wary -&gt; wary)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (trepidation -&gt; trepidation)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (surprising -&gt; surprising)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (superlative -&gt; superlative)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (sketchy -&gt; sketchy)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (slick -&gt; slick)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (rewarding -&gt; rewarding)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (nervousness -&gt; nervousness)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (mad -&gt; mad)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (inviting -&gt; inviting)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (cheesy -&gt; cheesy)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (admire -&gt; admire)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (mesmerized -&gt; mesmerized)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (unfortunate -&gt; unfortunate)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (stunningly -&gt; stunningly)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (stunned -&gt; stunned)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (stability -&gt; stability)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (raving -&gt; raving)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (quaint -&gt; quaint)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (wonderfull -&gt; wonderful)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (jealous -&gt; jealous)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (improving -&gt; improving)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (improvement -&gt; improvement)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (friendlier -&gt; friendlier)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (emotional -&gt; emotional)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (ecstatic -&gt; ecstatic)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (conscientious -&gt; conscientious)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (badly -&gt; badly)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (unspoiled -&gt; unspoiled)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (terribly -&gt; terribly)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (susceptible -&gt; susceptible)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (stuffed -&gt; stuffed)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (miserable -&gt; miserable)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (hassles -&gt; hassles)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (effortless -&gt; effortless)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (compliment -&gt; compliment)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (claustrophobia -&gt; claustrophobia)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (cheerfully -&gt; cheerfully)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (bummer -&gt; bummer)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (awkward -&gt; awkward)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (automatically -&gt; automatically)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (mindful -&gt; mindful)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (yummy -&gt; yummy)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (unstable -&gt; unstable)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (spoiled -&gt; spoiled)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (shocked -&gt; shocked)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (poorly -&gt; poorly)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (nerve -&gt; nerve)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (grace -&gt; grace)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (frustration -&gt; frustration)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (frightened -&gt; frightened)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (exhilaration -&gt; exhilaration)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (exhausted -&gt; exhausted)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (dissapointed -&gt; disappointed)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (cherished -&gt; cherish)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (annoyed -&gt; annoyed)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (strange -&gt; strange)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (reputable -&gt; reputable)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (ridiculous -&gt; ridiculous)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (rudely -&gt; rudely)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (serenity -&gt; serenity)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (relieved -&gt; relieved)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (suffered -&gt; suffered)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (unhappy -&gt; unhappy)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (unpleasant -&gt; unpleasant)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (powerful -&gt; powerful)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (worrying -&gt; worry)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (weird -&gt; weird)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (painful -&gt; painful)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (panic -&gt; panic)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (laughter -&gt; laughter)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (hopeful -&gt; hopeful)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (hesitating -&gt; hesitating)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (gushing -&gt; gushing)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (exhilerating -&gt; exhilarating)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (enthusiastically -&gt; enthusiastically)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (curious -&gt; curious)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (confusion -&gt; confusion)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (classy -&gt; classy)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (captivated -&gt; captivated)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (alas -&gt; alas)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (reassurance -&gt; reassurance)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (inspirational -&gt; inspirational)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (jovial -&gt; jovial)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (precision -&gt; precision)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (gratitude -&gt; gratitude)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (relief -&gt; relief)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (sublime -&gt; sublime)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (timid -&gt; timid)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (warmest -&gt; warmest)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (hug -&gt; hug)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (amaze -&gt; amaze)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (frightening -&gt; frightening)</t>
-  </si>
-  <si>
-    <t>1c. 语法变形拯救词 (calmer -&gt; calmer)</t>
-  </si>
-  <si>
-    <t>2a. 网络口语极级形容词 (Class 2 Gap)</t>
-  </si>
-  <si>
-    <t>2b. 低空观光领域专有词 (Class 3 Gap)</t>
+    <t>2a. Class 2 Web 2.0 Colloquial Superlatives (128 Words)</t>
+  </si>
+  <si>
+    <t>1a. Directly Mapped to NRC 8-Emotions (286 Words)</t>
+  </si>
+  <si>
+    <t>1b. Directly Mapped to Polarity Only (72 Words)</t>
+  </si>
+  <si>
+    <t>2b. Class 3 Low-Altitude Domain Lexicon (17 Words)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (concerned -&gt; concern)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (lucked -&gt; lucky)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (worries -&gt; worry)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (surprises -&gt; surprise)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (wonderfull -&gt; wonderful)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (dissapointed -&gt; disappointed)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (cherished -&gt; cherish)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (worrying -&gt; worry)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (suprise -&gt; surprise)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (marveled -&gt; marvel)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (hates -&gt; hate)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (hated -&gt; hate)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (suprised -&gt; surprised)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (regretting -&gt; regret)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (dreaded -&gt; dread)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (dreading -&gt; dread)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (horribly -&gt; horrible)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (scaring -&gt; scare)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (apprehensions -&gt; apprehension)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (aprehensive -&gt; apprehensive)</t>
+  </si>
+  <si>
+    <t>1c. Class 1 Morphological Rescued (disappointingly -&gt; disappointed)</t>
   </si>
 </sst>
 </file>
@@ -4631,7 +4313,7 @@
         <v>640</v>
       </c>
       <c r="E6" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -4648,7 +4330,7 @@
         <v>641</v>
       </c>
       <c r="E7" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -4835,7 +4517,7 @@
         <v>652</v>
       </c>
       <c r="E18" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -4886,7 +4568,7 @@
         <v>655</v>
       </c>
       <c r="E21" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -4903,7 +4585,7 @@
         <v>656</v>
       </c>
       <c r="E22" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -4937,7 +4619,7 @@
         <v>658</v>
       </c>
       <c r="E24" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -4971,7 +4653,7 @@
         <v>660</v>
       </c>
       <c r="E26" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -4988,7 +4670,7 @@
         <v>661</v>
       </c>
       <c r="E27" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -5005,7 +4687,7 @@
         <v>662</v>
       </c>
       <c r="E28" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -5022,7 +4704,7 @@
         <v>663</v>
       </c>
       <c r="E29" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -5039,7 +4721,7 @@
         <v>664</v>
       </c>
       <c r="E30" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -5056,7 +4738,7 @@
         <v>665</v>
       </c>
       <c r="E31" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -5073,7 +4755,7 @@
         <v>666</v>
       </c>
       <c r="E32" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -5175,7 +4857,7 @@
         <v>672</v>
       </c>
       <c r="E38" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -5226,7 +4908,7 @@
         <v>675</v>
       </c>
       <c r="E41" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -5311,7 +4993,7 @@
         <v>680</v>
       </c>
       <c r="E46" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -5328,7 +5010,7 @@
         <v>681</v>
       </c>
       <c r="E47" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -5413,7 +5095,7 @@
         <v>686</v>
       </c>
       <c r="E52" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -5447,7 +5129,7 @@
         <v>688</v>
       </c>
       <c r="E54" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -5498,7 +5180,7 @@
         <v>691</v>
       </c>
       <c r="E57" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -5549,7 +5231,7 @@
         <v>694</v>
       </c>
       <c r="E60" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -5566,7 +5248,7 @@
         <v>695</v>
       </c>
       <c r="E61" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -5600,7 +5282,7 @@
         <v>697</v>
       </c>
       <c r="E63" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -5685,7 +5367,7 @@
         <v>702</v>
       </c>
       <c r="E68" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -5702,7 +5384,7 @@
         <v>703</v>
       </c>
       <c r="E69" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -5787,7 +5469,7 @@
         <v>708</v>
       </c>
       <c r="E74" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -5804,7 +5486,7 @@
         <v>709</v>
       </c>
       <c r="E75" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -5838,7 +5520,7 @@
         <v>711</v>
       </c>
       <c r="E77" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -5855,7 +5537,7 @@
         <v>712</v>
       </c>
       <c r="E78" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -5889,7 +5571,7 @@
         <v>714</v>
       </c>
       <c r="E80" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -5923,7 +5605,7 @@
         <v>716</v>
       </c>
       <c r="E82" t="s">
-        <v>1255</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -5940,7 +5622,7 @@
         <v>717</v>
       </c>
       <c r="E83" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -5974,7 +5656,7 @@
         <v>719</v>
       </c>
       <c r="E85" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -5991,7 +5673,7 @@
         <v>720</v>
       </c>
       <c r="E86" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -6008,7 +5690,7 @@
         <v>716</v>
       </c>
       <c r="E87" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -6059,7 +5741,7 @@
         <v>723</v>
       </c>
       <c r="E90" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -6076,7 +5758,7 @@
         <v>724</v>
       </c>
       <c r="E91" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -6093,7 +5775,7 @@
         <v>725</v>
       </c>
       <c r="E92" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -6110,7 +5792,7 @@
         <v>726</v>
       </c>
       <c r="E93" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -6195,7 +5877,7 @@
         <v>731</v>
       </c>
       <c r="E98" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -6212,7 +5894,7 @@
         <v>732</v>
       </c>
       <c r="E99" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -6297,7 +5979,7 @@
         <v>737</v>
       </c>
       <c r="E104" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -6314,7 +5996,7 @@
         <v>738</v>
       </c>
       <c r="E105" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -6365,7 +6047,7 @@
         <v>741</v>
       </c>
       <c r="E108" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -6382,7 +6064,7 @@
         <v>742</v>
       </c>
       <c r="E109" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -6416,7 +6098,7 @@
         <v>744</v>
       </c>
       <c r="E111" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -6433,7 +6115,7 @@
         <v>745</v>
       </c>
       <c r="E112" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -6450,7 +6132,7 @@
         <v>746</v>
       </c>
       <c r="E113" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -6484,7 +6166,7 @@
         <v>748</v>
       </c>
       <c r="E115" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -6518,7 +6200,7 @@
         <v>750</v>
       </c>
       <c r="E117" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -6569,7 +6251,7 @@
         <v>753</v>
       </c>
       <c r="E120" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -6603,7 +6285,7 @@
         <v>755</v>
       </c>
       <c r="E122" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -6705,7 +6387,7 @@
         <v>761</v>
       </c>
       <c r="E128" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -6739,7 +6421,7 @@
         <v>763</v>
       </c>
       <c r="E130" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -6756,7 +6438,7 @@
         <v>764</v>
       </c>
       <c r="E131" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -6773,7 +6455,7 @@
         <v>765</v>
       </c>
       <c r="E132" t="s">
-        <v>1255</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -6875,7 +6557,7 @@
         <v>771</v>
       </c>
       <c r="E138" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -6892,7 +6574,7 @@
         <v>772</v>
       </c>
       <c r="E139" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -6909,7 +6591,7 @@
         <v>773</v>
       </c>
       <c r="E140" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -6926,7 +6608,7 @@
         <v>774</v>
       </c>
       <c r="E141" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -6943,7 +6625,7 @@
         <v>775</v>
       </c>
       <c r="E142" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -6960,7 +6642,7 @@
         <v>776</v>
       </c>
       <c r="E143" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -6977,7 +6659,7 @@
         <v>777</v>
       </c>
       <c r="E144" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -7062,7 +6744,7 @@
         <v>782</v>
       </c>
       <c r="E149" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -7147,7 +6829,7 @@
         <v>787</v>
       </c>
       <c r="E154" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -7164,7 +6846,7 @@
         <v>788</v>
       </c>
       <c r="E155" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -7181,7 +6863,7 @@
         <v>789</v>
       </c>
       <c r="E156" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -7215,7 +6897,7 @@
         <v>791</v>
       </c>
       <c r="E158" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -7266,7 +6948,7 @@
         <v>794</v>
       </c>
       <c r="E161" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -7300,7 +6982,7 @@
         <v>796</v>
       </c>
       <c r="E163" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -7317,7 +6999,7 @@
         <v>797</v>
       </c>
       <c r="E164" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -7351,7 +7033,7 @@
         <v>799</v>
       </c>
       <c r="E166" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -7368,7 +7050,7 @@
         <v>800</v>
       </c>
       <c r="E167" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -7385,7 +7067,7 @@
         <v>801</v>
       </c>
       <c r="E168" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -7402,7 +7084,7 @@
         <v>802</v>
       </c>
       <c r="E169" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -7453,7 +7135,7 @@
         <v>805</v>
       </c>
       <c r="E172" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -7470,7 +7152,7 @@
         <v>806</v>
       </c>
       <c r="E173" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -7555,7 +7237,7 @@
         <v>811</v>
       </c>
       <c r="E178" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -7572,7 +7254,7 @@
         <v>812</v>
       </c>
       <c r="E179" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -7589,7 +7271,7 @@
         <v>813</v>
       </c>
       <c r="E180" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="181" spans="1:5">
@@ -7606,7 +7288,7 @@
         <v>772</v>
       </c>
       <c r="E181" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="182" spans="1:5">
@@ -7623,7 +7305,7 @@
         <v>814</v>
       </c>
       <c r="E182" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="183" spans="1:5">
@@ -7657,7 +7339,7 @@
         <v>816</v>
       </c>
       <c r="E184" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="185" spans="1:5">
@@ -7674,7 +7356,7 @@
         <v>817</v>
       </c>
       <c r="E185" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -7691,7 +7373,7 @@
         <v>818</v>
       </c>
       <c r="E186" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="187" spans="1:5">
@@ -7708,7 +7390,7 @@
         <v>819</v>
       </c>
       <c r="E187" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -7725,7 +7407,7 @@
         <v>820</v>
       </c>
       <c r="E188" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="189" spans="1:5">
@@ -7742,7 +7424,7 @@
         <v>821</v>
       </c>
       <c r="E189" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -7776,7 +7458,7 @@
         <v>823</v>
       </c>
       <c r="E191" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -7793,7 +7475,7 @@
         <v>824</v>
       </c>
       <c r="E192" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -7861,7 +7543,7 @@
         <v>828</v>
       </c>
       <c r="E196" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -7963,7 +7645,7 @@
         <v>727</v>
       </c>
       <c r="E202" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -7980,7 +7662,7 @@
         <v>834</v>
       </c>
       <c r="E203" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -8014,7 +7696,7 @@
         <v>836</v>
       </c>
       <c r="E205" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -8065,7 +7747,7 @@
         <v>839</v>
       </c>
       <c r="E208" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -8116,7 +7798,7 @@
         <v>842</v>
       </c>
       <c r="E211" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -8133,7 +7815,7 @@
         <v>843</v>
       </c>
       <c r="E212" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -8218,7 +7900,7 @@
         <v>848</v>
       </c>
       <c r="E217" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -8286,7 +7968,7 @@
         <v>852</v>
       </c>
       <c r="E221" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -8303,7 +7985,7 @@
         <v>853</v>
       </c>
       <c r="E222" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -8320,7 +8002,7 @@
         <v>854</v>
       </c>
       <c r="E223" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -8337,7 +8019,7 @@
         <v>855</v>
       </c>
       <c r="E224" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -8371,7 +8053,7 @@
         <v>857</v>
       </c>
       <c r="E226" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -8439,7 +8121,7 @@
         <v>861</v>
       </c>
       <c r="E230" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -8490,7 +8172,7 @@
         <v>864</v>
       </c>
       <c r="E233" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -8507,7 +8189,7 @@
         <v>865</v>
       </c>
       <c r="E234" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -8524,7 +8206,7 @@
         <v>866</v>
       </c>
       <c r="E235" t="s">
-        <v>1255</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -8592,7 +8274,7 @@
         <v>870</v>
       </c>
       <c r="E239" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="240" spans="1:5">
@@ -8609,7 +8291,7 @@
         <v>871</v>
       </c>
       <c r="E240" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="241" spans="1:5">
@@ -8626,7 +8308,7 @@
         <v>872</v>
       </c>
       <c r="E241" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -8643,7 +8325,7 @@
         <v>873</v>
       </c>
       <c r="E242" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="243" spans="1:5">
@@ -8677,7 +8359,7 @@
         <v>874</v>
       </c>
       <c r="E244" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="245" spans="1:5">
@@ -8694,7 +8376,7 @@
         <v>875</v>
       </c>
       <c r="E245" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="246" spans="1:5">
@@ -8711,7 +8393,7 @@
         <v>876</v>
       </c>
       <c r="E246" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="247" spans="1:5">
@@ -8728,7 +8410,7 @@
         <v>682</v>
       </c>
       <c r="E247" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="248" spans="1:5">
@@ -8745,7 +8427,7 @@
         <v>877</v>
       </c>
       <c r="E248" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="249" spans="1:5">
@@ -8762,7 +8444,7 @@
         <v>878</v>
       </c>
       <c r="E249" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="250" spans="1:5">
@@ -8779,7 +8461,7 @@
         <v>879</v>
       </c>
       <c r="E250" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="251" spans="1:5">
@@ -8796,7 +8478,7 @@
         <v>880</v>
       </c>
       <c r="E251" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="252" spans="1:5">
@@ -8813,7 +8495,7 @@
         <v>881</v>
       </c>
       <c r="E252" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="253" spans="1:5">
@@ -8830,7 +8512,7 @@
         <v>882</v>
       </c>
       <c r="E253" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="254" spans="1:5">
@@ -8847,7 +8529,7 @@
         <v>883</v>
       </c>
       <c r="E254" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="255" spans="1:5">
@@ -8864,7 +8546,7 @@
         <v>884</v>
       </c>
       <c r="E255" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="256" spans="1:5">
@@ -8898,7 +8580,7 @@
         <v>886</v>
       </c>
       <c r="E257" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="258" spans="1:5">
@@ -8915,7 +8597,7 @@
         <v>887</v>
       </c>
       <c r="E258" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="259" spans="1:5">
@@ -8949,7 +8631,7 @@
         <v>889</v>
       </c>
       <c r="E260" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="261" spans="1:5">
@@ -8983,7 +8665,7 @@
         <v>891</v>
       </c>
       <c r="E262" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="263" spans="1:5">
@@ -9017,7 +8699,7 @@
         <v>893</v>
       </c>
       <c r="E264" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="265" spans="1:5">
@@ -9068,7 +8750,7 @@
         <v>896</v>
       </c>
       <c r="E267" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="268" spans="1:5">
@@ -9119,7 +8801,7 @@
         <v>899</v>
       </c>
       <c r="E270" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="271" spans="1:5">
@@ -9136,7 +8818,7 @@
         <v>900</v>
       </c>
       <c r="E271" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="272" spans="1:5">
@@ -9153,7 +8835,7 @@
         <v>901</v>
       </c>
       <c r="E272" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="273" spans="1:5">
@@ -9221,7 +8903,7 @@
         <v>905</v>
       </c>
       <c r="E276" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="277" spans="1:5">
@@ -9238,7 +8920,7 @@
         <v>906</v>
       </c>
       <c r="E277" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="278" spans="1:5">
@@ -9255,7 +8937,7 @@
         <v>907</v>
       </c>
       <c r="E278" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="279" spans="1:5">
@@ -9306,7 +8988,7 @@
         <v>909</v>
       </c>
       <c r="E281" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="282" spans="1:5">
@@ -9340,7 +9022,7 @@
         <v>911</v>
       </c>
       <c r="E283" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="284" spans="1:5">
@@ -9374,7 +9056,7 @@
         <v>913</v>
       </c>
       <c r="E285" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="286" spans="1:5">
@@ -9391,7 +9073,7 @@
         <v>914</v>
       </c>
       <c r="E286" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="287" spans="1:5">
@@ -9408,7 +9090,7 @@
         <v>915</v>
       </c>
       <c r="E287" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="288" spans="1:5">
@@ -9425,7 +9107,7 @@
         <v>916</v>
       </c>
       <c r="E288" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="289" spans="1:5">
@@ -9442,7 +9124,7 @@
         <v>917</v>
       </c>
       <c r="E289" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="290" spans="1:5">
@@ -9459,7 +9141,7 @@
         <v>918</v>
       </c>
       <c r="E290" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="291" spans="1:5">
@@ -9527,7 +9209,7 @@
         <v>922</v>
       </c>
       <c r="E294" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="295" spans="1:5">
@@ -9578,7 +9260,7 @@
         <v>901</v>
       </c>
       <c r="E297" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="298" spans="1:5">
@@ -9595,7 +9277,7 @@
         <v>925</v>
       </c>
       <c r="E298" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="299" spans="1:5">
@@ -9629,7 +9311,7 @@
         <v>927</v>
       </c>
       <c r="E300" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="301" spans="1:5">
@@ -9646,7 +9328,7 @@
         <v>928</v>
       </c>
       <c r="E301" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="302" spans="1:5">
@@ -9663,7 +9345,7 @@
         <v>929</v>
       </c>
       <c r="E302" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="303" spans="1:5">
@@ -9697,7 +9379,7 @@
         <v>931</v>
       </c>
       <c r="E304" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="305" spans="1:5">
@@ -9731,7 +9413,7 @@
         <v>933</v>
       </c>
       <c r="E306" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="307" spans="1:5">
@@ -9748,7 +9430,7 @@
         <v>934</v>
       </c>
       <c r="E307" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="308" spans="1:5">
@@ -9765,7 +9447,7 @@
         <v>935</v>
       </c>
       <c r="E308" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="309" spans="1:5">
@@ -9782,7 +9464,7 @@
         <v>936</v>
       </c>
       <c r="E309" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="310" spans="1:5">
@@ -9816,7 +9498,7 @@
         <v>938</v>
       </c>
       <c r="E311" t="s">
-        <v>1256</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="312" spans="1:5">
@@ -9833,7 +9515,7 @@
         <v>939</v>
       </c>
       <c r="E312" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="313" spans="1:5">
@@ -9867,7 +9549,7 @@
         <v>941</v>
       </c>
       <c r="E314" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="315" spans="1:5">
@@ -9884,7 +9566,7 @@
         <v>942</v>
       </c>
       <c r="E315" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="316" spans="1:5">
@@ -9935,7 +9617,7 @@
         <v>945</v>
       </c>
       <c r="E318" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="319" spans="1:5">
@@ -9969,7 +9651,7 @@
         <v>947</v>
       </c>
       <c r="E320" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="321" spans="1:5">
@@ -10003,7 +9685,7 @@
         <v>949</v>
       </c>
       <c r="E322" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="323" spans="1:5">
@@ -10020,7 +9702,7 @@
         <v>950</v>
       </c>
       <c r="E323" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="324" spans="1:5">
@@ -10037,7 +9719,7 @@
         <v>951</v>
       </c>
       <c r="E324" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="325" spans="1:5">
@@ -10054,7 +9736,7 @@
         <v>952</v>
       </c>
       <c r="E325" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="326" spans="1:5">
@@ -10071,7 +9753,7 @@
         <v>953</v>
       </c>
       <c r="E326" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="327" spans="1:5">
@@ -10088,7 +9770,7 @@
         <v>954</v>
       </c>
       <c r="E327" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="328" spans="1:5">
@@ -10173,7 +9855,7 @@
         <v>959</v>
       </c>
       <c r="E332" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="333" spans="1:5">
@@ -10207,7 +9889,7 @@
         <v>961</v>
       </c>
       <c r="E334" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="335" spans="1:5">
@@ -10224,7 +9906,7 @@
         <v>962</v>
       </c>
       <c r="E335" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="336" spans="1:5">
@@ -10241,7 +9923,7 @@
         <v>963</v>
       </c>
       <c r="E336" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="337" spans="1:5">
@@ -10275,7 +9957,7 @@
         <v>965</v>
       </c>
       <c r="E338" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="339" spans="1:5">
@@ -10292,7 +9974,7 @@
         <v>966</v>
       </c>
       <c r="E339" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="340" spans="1:5">
@@ -10309,7 +9991,7 @@
         <v>967</v>
       </c>
       <c r="E340" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="341" spans="1:5">
@@ -10326,7 +10008,7 @@
         <v>968</v>
       </c>
       <c r="E341" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="342" spans="1:5">
@@ -10360,7 +10042,7 @@
         <v>830</v>
       </c>
       <c r="E343" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="344" spans="1:5">
@@ -10394,7 +10076,7 @@
         <v>971</v>
       </c>
       <c r="E345" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="346" spans="1:5">
@@ -10411,7 +10093,7 @@
         <v>972</v>
       </c>
       <c r="E346" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="347" spans="1:5">
@@ -10445,7 +10127,7 @@
         <v>974</v>
       </c>
       <c r="E348" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="349" spans="1:5">
@@ -10462,7 +10144,7 @@
         <v>975</v>
       </c>
       <c r="E349" t="s">
-        <v>1256</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="350" spans="1:5">
@@ -10615,7 +10297,7 @@
         <v>984</v>
       </c>
       <c r="E358" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="359" spans="1:5">
@@ -10632,7 +10314,7 @@
         <v>985</v>
       </c>
       <c r="E359" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="360" spans="1:5">
@@ -10649,7 +10331,7 @@
         <v>986</v>
       </c>
       <c r="E360" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="361" spans="1:5">
@@ -10666,7 +10348,7 @@
         <v>987</v>
       </c>
       <c r="E361" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="362" spans="1:5">
@@ -10683,7 +10365,7 @@
         <v>988</v>
       </c>
       <c r="E362" t="s">
-        <v>1259</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="363" spans="1:5">
@@ -10700,7 +10382,7 @@
         <v>989</v>
       </c>
       <c r="E363" t="s">
-        <v>1260</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="364" spans="1:5">
@@ -10717,7 +10399,7 @@
         <v>990</v>
       </c>
       <c r="E364" t="s">
-        <v>1261</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="365" spans="1:5">
@@ -10734,7 +10416,7 @@
         <v>991</v>
       </c>
       <c r="E365" t="s">
-        <v>1262</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="366" spans="1:5">
@@ -10751,7 +10433,7 @@
         <v>992</v>
       </c>
       <c r="E366" t="s">
-        <v>1263</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="367" spans="1:5">
@@ -10768,7 +10450,7 @@
         <v>993</v>
       </c>
       <c r="E367" t="s">
-        <v>1264</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="368" spans="1:5">
@@ -10785,7 +10467,7 @@
         <v>994</v>
       </c>
       <c r="E368" t="s">
-        <v>1265</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="369" spans="1:5">
@@ -10802,7 +10484,7 @@
         <v>995</v>
       </c>
       <c r="E369" t="s">
-        <v>1266</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="370" spans="1:5">
@@ -10819,7 +10501,7 @@
         <v>996</v>
       </c>
       <c r="E370" t="s">
-        <v>1267</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="371" spans="1:5">
@@ -10836,7 +10518,7 @@
         <v>997</v>
       </c>
       <c r="E371" t="s">
-        <v>1268</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="372" spans="1:5">
@@ -10853,7 +10535,7 @@
         <v>998</v>
       </c>
       <c r="E372" t="s">
-        <v>1269</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="373" spans="1:5">
@@ -10870,7 +10552,7 @@
         <v>999</v>
       </c>
       <c r="E373" t="s">
-        <v>1270</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="374" spans="1:5">
@@ -10887,7 +10569,7 @@
         <v>1000</v>
       </c>
       <c r="E374" t="s">
-        <v>1271</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="375" spans="1:5">
@@ -10904,7 +10586,7 @@
         <v>1001</v>
       </c>
       <c r="E375" t="s">
-        <v>1272</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="376" spans="1:5">
@@ -10921,7 +10603,7 @@
         <v>1002</v>
       </c>
       <c r="E376" t="s">
-        <v>1273</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="377" spans="1:5">
@@ -10938,7 +10620,7 @@
         <v>1003</v>
       </c>
       <c r="E377" t="s">
-        <v>1274</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="378" spans="1:5">
@@ -10955,7 +10637,7 @@
         <v>1004</v>
       </c>
       <c r="E378" t="s">
-        <v>1275</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="379" spans="1:5">
@@ -10972,7 +10654,7 @@
         <v>1005</v>
       </c>
       <c r="E379" t="s">
-        <v>1276</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="380" spans="1:5">
@@ -10989,7 +10671,7 @@
         <v>1006</v>
       </c>
       <c r="E380" t="s">
-        <v>1277</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="381" spans="1:5">
@@ -11006,7 +10688,7 @@
         <v>1007</v>
       </c>
       <c r="E381" t="s">
-        <v>1278</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="382" spans="1:5">
@@ -11023,7 +10705,7 @@
         <v>1008</v>
       </c>
       <c r="E382" t="s">
-        <v>1279</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="383" spans="1:5">
@@ -11040,7 +10722,7 @@
         <v>1009</v>
       </c>
       <c r="E383" t="s">
-        <v>1280</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="384" spans="1:5">
@@ -11057,7 +10739,7 @@
         <v>1010</v>
       </c>
       <c r="E384" t="s">
-        <v>1281</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="385" spans="1:5">
@@ -11074,7 +10756,7 @@
         <v>1011</v>
       </c>
       <c r="E385" t="s">
-        <v>1282</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="386" spans="1:5">
@@ -11091,7 +10773,7 @@
         <v>1012</v>
       </c>
       <c r="E386" t="s">
-        <v>1283</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="387" spans="1:5">
@@ -11108,7 +10790,7 @@
         <v>1013</v>
       </c>
       <c r="E387" t="s">
-        <v>1284</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="388" spans="1:5">
@@ -11125,7 +10807,7 @@
         <v>1014</v>
       </c>
       <c r="E388" t="s">
-        <v>1285</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="389" spans="1:5">
@@ -11142,7 +10824,7 @@
         <v>1015</v>
       </c>
       <c r="E389" t="s">
-        <v>1286</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="390" spans="1:5">
@@ -11159,7 +10841,7 @@
         <v>1016</v>
       </c>
       <c r="E390" t="s">
-        <v>1287</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="391" spans="1:5">
@@ -11176,7 +10858,7 @@
         <v>1017</v>
       </c>
       <c r="E391" t="s">
-        <v>1288</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="392" spans="1:5">
@@ -11193,7 +10875,7 @@
         <v>1018</v>
       </c>
       <c r="E392" t="s">
-        <v>1289</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="393" spans="1:5">
@@ -11210,7 +10892,7 @@
         <v>1019</v>
       </c>
       <c r="E393" t="s">
-        <v>1290</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="394" spans="1:5">
@@ -11227,7 +10909,7 @@
         <v>1020</v>
       </c>
       <c r="E394" t="s">
-        <v>1291</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="395" spans="1:5">
@@ -11244,7 +10926,7 @@
         <v>1021</v>
       </c>
       <c r="E395" t="s">
-        <v>1292</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="396" spans="1:5">
@@ -11261,7 +10943,7 @@
         <v>1022</v>
       </c>
       <c r="E396" t="s">
-        <v>1293</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="397" spans="1:5">
@@ -11278,7 +10960,7 @@
         <v>1023</v>
       </c>
       <c r="E397" t="s">
-        <v>1294</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="398" spans="1:5">
@@ -11295,7 +10977,7 @@
         <v>1024</v>
       </c>
       <c r="E398" t="s">
-        <v>1295</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="399" spans="1:5">
@@ -11312,7 +10994,7 @@
         <v>1025</v>
       </c>
       <c r="E399" t="s">
-        <v>1296</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="400" spans="1:5">
@@ -11329,7 +11011,7 @@
         <v>1026</v>
       </c>
       <c r="E400" t="s">
-        <v>1297</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="401" spans="1:5">
@@ -11346,7 +11028,7 @@
         <v>1027</v>
       </c>
       <c r="E401" t="s">
-        <v>1298</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="402" spans="1:5">
@@ -11363,7 +11045,7 @@
         <v>1028</v>
       </c>
       <c r="E402" t="s">
-        <v>1299</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="403" spans="1:5">
@@ -11380,7 +11062,7 @@
         <v>1029</v>
       </c>
       <c r="E403" t="s">
-        <v>1300</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="404" spans="1:5">
@@ -11397,7 +11079,7 @@
         <v>1030</v>
       </c>
       <c r="E404" t="s">
-        <v>1301</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="405" spans="1:5">
@@ -11414,7 +11096,7 @@
         <v>1031</v>
       </c>
       <c r="E405" t="s">
-        <v>1302</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="406" spans="1:5">
@@ -11431,7 +11113,7 @@
         <v>1032</v>
       </c>
       <c r="E406" t="s">
-        <v>1303</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="407" spans="1:5">
@@ -11448,7 +11130,7 @@
         <v>1033</v>
       </c>
       <c r="E407" t="s">
-        <v>1304</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="408" spans="1:5">
@@ -11465,7 +11147,7 @@
         <v>1034</v>
       </c>
       <c r="E408" t="s">
-        <v>1305</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="409" spans="1:5">
@@ -11482,7 +11164,7 @@
         <v>1035</v>
       </c>
       <c r="E409" t="s">
-        <v>1306</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="410" spans="1:5">
@@ -11499,7 +11181,7 @@
         <v>1036</v>
       </c>
       <c r="E410" t="s">
-        <v>1307</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="411" spans="1:5">
@@ -11516,7 +11198,7 @@
         <v>1037</v>
       </c>
       <c r="E411" t="s">
-        <v>1308</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="412" spans="1:5">
@@ -11533,7 +11215,7 @@
         <v>1038</v>
       </c>
       <c r="E412" t="s">
-        <v>1309</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="413" spans="1:5">
@@ -11550,7 +11232,7 @@
         <v>1039</v>
       </c>
       <c r="E413" t="s">
-        <v>1310</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="414" spans="1:5">
@@ -11567,7 +11249,7 @@
         <v>1040</v>
       </c>
       <c r="E414" t="s">
-        <v>1311</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="415" spans="1:5">
@@ -11584,7 +11266,7 @@
         <v>1041</v>
       </c>
       <c r="E415" t="s">
-        <v>1312</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="416" spans="1:5">
@@ -11601,7 +11283,7 @@
         <v>1042</v>
       </c>
       <c r="E416" t="s">
-        <v>1313</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="417" spans="1:5">
@@ -11618,7 +11300,7 @@
         <v>1043</v>
       </c>
       <c r="E417" t="s">
-        <v>1314</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="418" spans="1:5">
@@ -11635,7 +11317,7 @@
         <v>1044</v>
       </c>
       <c r="E418" t="s">
-        <v>1315</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="419" spans="1:5">
@@ -11652,7 +11334,7 @@
         <v>1045</v>
       </c>
       <c r="E419" t="s">
-        <v>1316</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="420" spans="1:5">
@@ -11669,7 +11351,7 @@
         <v>1046</v>
       </c>
       <c r="E420" t="s">
-        <v>1317</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="421" spans="1:5">
@@ -11686,7 +11368,7 @@
         <v>1047</v>
       </c>
       <c r="E421" t="s">
-        <v>1318</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="422" spans="1:5">
@@ -11703,7 +11385,7 @@
         <v>1048</v>
       </c>
       <c r="E422" t="s">
-        <v>1319</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="423" spans="1:5">
@@ -11720,7 +11402,7 @@
         <v>1049</v>
       </c>
       <c r="E423" t="s">
-        <v>1320</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="424" spans="1:5">
@@ -11737,7 +11419,7 @@
         <v>1050</v>
       </c>
       <c r="E424" t="s">
-        <v>1321</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="425" spans="1:5">
@@ -11754,7 +11436,7 @@
         <v>1051</v>
       </c>
       <c r="E425" t="s">
-        <v>1322</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="426" spans="1:5">
@@ -11771,7 +11453,7 @@
         <v>1052</v>
       </c>
       <c r="E426" t="s">
-        <v>1323</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="427" spans="1:5">
@@ -11788,7 +11470,7 @@
         <v>1053</v>
       </c>
       <c r="E427" t="s">
-        <v>1324</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="428" spans="1:5">
@@ -11805,7 +11487,7 @@
         <v>1054</v>
       </c>
       <c r="E428" t="s">
-        <v>1325</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="429" spans="1:5">
@@ -11822,7 +11504,7 @@
         <v>1055</v>
       </c>
       <c r="E429" t="s">
-        <v>1326</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="430" spans="1:5">
@@ -11839,7 +11521,7 @@
         <v>1056</v>
       </c>
       <c r="E430" t="s">
-        <v>1327</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="431" spans="1:5">
@@ -11856,7 +11538,7 @@
         <v>1057</v>
       </c>
       <c r="E431" t="s">
-        <v>1328</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="432" spans="1:5">
@@ -11873,7 +11555,7 @@
         <v>1058</v>
       </c>
       <c r="E432" t="s">
-        <v>1329</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="433" spans="1:5">
@@ -11890,7 +11572,7 @@
         <v>1059</v>
       </c>
       <c r="E433" t="s">
-        <v>1330</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="434" spans="1:5">
@@ -11907,7 +11589,7 @@
         <v>1060</v>
       </c>
       <c r="E434" t="s">
-        <v>1331</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="435" spans="1:5">
@@ -11924,7 +11606,7 @@
         <v>870</v>
       </c>
       <c r="E435" t="s">
-        <v>1332</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="436" spans="1:5">
@@ -11941,7 +11623,7 @@
         <v>1061</v>
       </c>
       <c r="E436" t="s">
-        <v>1333</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="437" spans="1:5">
@@ -11958,7 +11640,7 @@
         <v>1062</v>
       </c>
       <c r="E437" t="s">
-        <v>1334</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="438" spans="1:5">
@@ -11975,7 +11657,7 @@
         <v>1063</v>
       </c>
       <c r="E438" t="s">
-        <v>1335</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="439" spans="1:5">
@@ -11992,7 +11674,7 @@
         <v>1064</v>
       </c>
       <c r="E439" t="s">
-        <v>1336</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="440" spans="1:5">
@@ -12009,7 +11691,7 @@
         <v>1065</v>
       </c>
       <c r="E440" t="s">
-        <v>1337</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="441" spans="1:5">
@@ -12026,7 +11708,7 @@
         <v>1066</v>
       </c>
       <c r="E441" t="s">
-        <v>1338</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="442" spans="1:5">
@@ -12043,7 +11725,7 @@
         <v>1067</v>
       </c>
       <c r="E442" t="s">
-        <v>1339</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="443" spans="1:5">
@@ -12060,7 +11742,7 @@
         <v>1068</v>
       </c>
       <c r="E443" t="s">
-        <v>1340</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="444" spans="1:5">
@@ -12077,7 +11759,7 @@
         <v>1069</v>
       </c>
       <c r="E444" t="s">
-        <v>1341</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="445" spans="1:5">
@@ -12094,7 +11776,7 @@
         <v>1070</v>
       </c>
       <c r="E445" t="s">
-        <v>1342</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="446" spans="1:5">
@@ -12111,7 +11793,7 @@
         <v>1071</v>
       </c>
       <c r="E446" t="s">
-        <v>1343</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="447" spans="1:5">
@@ -12128,7 +11810,7 @@
         <v>1072</v>
       </c>
       <c r="E447" t="s">
-        <v>1344</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="448" spans="1:5">
@@ -12145,7 +11827,7 @@
         <v>1073</v>
       </c>
       <c r="E448" t="s">
-        <v>1345</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="449" spans="1:5">
@@ -12162,7 +11844,7 @@
         <v>1074</v>
       </c>
       <c r="E449" t="s">
-        <v>1346</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="450" spans="1:5">
@@ -12179,7 +11861,7 @@
         <v>1075</v>
       </c>
       <c r="E450" t="s">
-        <v>1347</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="451" spans="1:5">
@@ -12196,7 +11878,7 @@
         <v>1076</v>
       </c>
       <c r="E451" t="s">
-        <v>1348</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="452" spans="1:5">
@@ -12213,7 +11895,7 @@
         <v>1077</v>
       </c>
       <c r="E452" t="s">
-        <v>1349</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="453" spans="1:5">
@@ -12230,7 +11912,7 @@
         <v>1078</v>
       </c>
       <c r="E453" t="s">
-        <v>1350</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="454" spans="1:5">
@@ -12247,7 +11929,7 @@
         <v>1079</v>
       </c>
       <c r="E454" t="s">
-        <v>1351</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="455" spans="1:5">
@@ -12264,7 +11946,7 @@
         <v>1080</v>
       </c>
       <c r="E455" t="s">
-        <v>1352</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="456" spans="1:5">
@@ -12281,7 +11963,7 @@
         <v>1081</v>
       </c>
       <c r="E456" t="s">
-        <v>1353</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="457" spans="1:5">
@@ -12298,7 +11980,7 @@
         <v>1082</v>
       </c>
       <c r="E457" t="s">
-        <v>1354</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="458" spans="1:5">
@@ -12315,7 +11997,7 @@
         <v>1083</v>
       </c>
       <c r="E458" t="s">
-        <v>1355</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="459" spans="1:5">
@@ -12332,7 +12014,7 @@
         <v>1084</v>
       </c>
       <c r="E459" t="s">
-        <v>1356</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="460" spans="1:5">
@@ -12349,7 +12031,7 @@
         <v>1085</v>
       </c>
       <c r="E460" t="s">
-        <v>1357</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="461" spans="1:5">
@@ -12366,7 +12048,7 @@
         <v>1086</v>
       </c>
       <c r="E461" t="s">
-        <v>1358</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="462" spans="1:5">
@@ -12383,7 +12065,7 @@
         <v>1087</v>
       </c>
       <c r="E462" t="s">
-        <v>1359</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="463" spans="1:5">
@@ -12400,7 +12082,7 @@
         <v>1088</v>
       </c>
       <c r="E463" t="s">
-        <v>1360</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="464" spans="1:5">
@@ -12417,7 +12099,7 @@
         <v>1089</v>
       </c>
       <c r="E464" t="s">
-        <v>1361</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="465" spans="1:5">
@@ -12434,7 +12116,7 @@
         <v>1090</v>
       </c>
       <c r="E465" t="s">
-        <v>1362</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="466" spans="1:5">
@@ -12451,7 +12133,7 @@
         <v>1091</v>
       </c>
       <c r="E466" t="s">
-        <v>1363</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="467" spans="1:5">
@@ -12468,7 +12150,7 @@
         <v>1092</v>
       </c>
       <c r="E467" t="s">
-        <v>1364</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="468" spans="1:5">
@@ -12485,7 +12167,7 @@
         <v>1093</v>
       </c>
       <c r="E468" t="s">
-        <v>1365</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="469" spans="1:5">
@@ -12502,7 +12184,7 @@
         <v>1094</v>
       </c>
       <c r="E469" t="s">
-        <v>1366</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="470" spans="1:5">
@@ -12519,7 +12201,7 @@
         <v>1095</v>
       </c>
       <c r="E470" t="s">
-        <v>1367</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="471" spans="1:5">
@@ -12536,7 +12218,7 @@
         <v>1096</v>
       </c>
       <c r="E471" t="s">
-        <v>1368</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="472" spans="1:5">
@@ -12553,7 +12235,7 @@
         <v>1097</v>
       </c>
       <c r="E472" t="s">
-        <v>1369</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="473" spans="1:5">
@@ -12570,7 +12252,7 @@
         <v>1098</v>
       </c>
       <c r="E473" t="s">
-        <v>1370</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="474" spans="1:5">
@@ -12587,7 +12269,7 @@
         <v>1099</v>
       </c>
       <c r="E474" t="s">
-        <v>1371</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="475" spans="1:5">
@@ -12604,7 +12286,7 @@
         <v>1100</v>
       </c>
       <c r="E475" t="s">
-        <v>1372</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="476" spans="1:5">
@@ -12621,7 +12303,7 @@
         <v>1101</v>
       </c>
       <c r="E476" t="s">
-        <v>1373</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="477" spans="1:5">
@@ -12638,7 +12320,7 @@
         <v>1102</v>
       </c>
       <c r="E477" t="s">
-        <v>1374</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="478" spans="1:5">
@@ -12655,7 +12337,7 @@
         <v>1103</v>
       </c>
       <c r="E478" t="s">
-        <v>1375</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="479" spans="1:5">
@@ -12672,7 +12354,7 @@
         <v>1104</v>
       </c>
       <c r="E479" t="s">
-        <v>1376</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="480" spans="1:5">
@@ -12689,7 +12371,7 @@
         <v>1105</v>
       </c>
       <c r="E480" t="s">
-        <v>1377</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="481" spans="1:5">
@@ -12706,7 +12388,7 @@
         <v>1106</v>
       </c>
       <c r="E481" t="s">
-        <v>1378</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="482" spans="1:5">
@@ -12723,7 +12405,7 @@
         <v>1107</v>
       </c>
       <c r="E482" t="s">
-        <v>1379</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="483" spans="1:5">
@@ -12740,7 +12422,7 @@
         <v>1108</v>
       </c>
       <c r="E483" t="s">
-        <v>1380</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="484" spans="1:5">
@@ -12757,7 +12439,7 @@
         <v>1109</v>
       </c>
       <c r="E484" t="s">
-        <v>1381</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="485" spans="1:5">
@@ -12774,7 +12456,7 @@
         <v>1110</v>
       </c>
       <c r="E485" t="s">
-        <v>1382</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="486" spans="1:5">
@@ -12791,7 +12473,7 @@
         <v>1111</v>
       </c>
       <c r="E486" t="s">
-        <v>1383</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="487" spans="1:5">
@@ -12808,7 +12490,7 @@
         <v>1112</v>
       </c>
       <c r="E487" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="488" spans="1:5">
@@ -12825,7 +12507,7 @@
         <v>1113</v>
       </c>
       <c r="E488" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="489" spans="1:5">
@@ -12842,7 +12524,7 @@
         <v>1114</v>
       </c>
       <c r="E489" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="490" spans="1:5">
@@ -12859,7 +12541,7 @@
         <v>1115</v>
       </c>
       <c r="E490" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="491" spans="1:5">
@@ -12876,7 +12558,7 @@
         <v>1116</v>
       </c>
       <c r="E491" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="492" spans="1:5">
@@ -12893,7 +12575,7 @@
         <v>1117</v>
       </c>
       <c r="E492" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="493" spans="1:5">
@@ -12910,7 +12592,7 @@
         <v>1031</v>
       </c>
       <c r="E493" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="494" spans="1:5">
@@ -12927,7 +12609,7 @@
         <v>1118</v>
       </c>
       <c r="E494" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="495" spans="1:5">
@@ -12944,7 +12626,7 @@
         <v>1119</v>
       </c>
       <c r="E495" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="496" spans="1:5">
@@ -12961,7 +12643,7 @@
         <v>1120</v>
       </c>
       <c r="E496" t="s">
-        <v>1384</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="497" spans="1:5">
@@ -12978,7 +12660,7 @@
         <v>1121</v>
       </c>
       <c r="E497" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="498" spans="1:5">
@@ -12995,7 +12677,7 @@
         <v>1122</v>
       </c>
       <c r="E498" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="499" spans="1:5">
@@ -13012,7 +12694,7 @@
         <v>1123</v>
       </c>
       <c r="E499" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="500" spans="1:5">
@@ -13029,7 +12711,7 @@
         <v>1124</v>
       </c>
       <c r="E500" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="501" spans="1:5">
@@ -13046,7 +12728,7 @@
         <v>1125</v>
       </c>
       <c r="E501" t="s">
-        <v>1384</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="502" spans="1:5">
@@ -13063,7 +12745,7 @@
         <v>1126</v>
       </c>
       <c r="E502" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="503" spans="1:5">
@@ -13080,7 +12762,7 @@
         <v>1127</v>
       </c>
       <c r="E503" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="504" spans="1:5">
@@ -13097,7 +12779,7 @@
         <v>1128</v>
       </c>
       <c r="E504" t="s">
-        <v>1384</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="505" spans="1:5">
@@ -13114,7 +12796,7 @@
         <v>1129</v>
       </c>
       <c r="E505" t="s">
-        <v>1384</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="506" spans="1:5">
@@ -13131,7 +12813,7 @@
         <v>1130</v>
       </c>
       <c r="E506" t="s">
-        <v>1384</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="507" spans="1:5">
@@ -13148,7 +12830,7 @@
         <v>1131</v>
       </c>
       <c r="E507" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="508" spans="1:5">
@@ -13165,7 +12847,7 @@
         <v>1132</v>
       </c>
       <c r="E508" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="509" spans="1:5">
@@ -13182,7 +12864,7 @@
         <v>1133</v>
       </c>
       <c r="E509" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="510" spans="1:5">
@@ -13199,7 +12881,7 @@
         <v>1134</v>
       </c>
       <c r="E510" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="511" spans="1:5">
@@ -13216,7 +12898,7 @@
         <v>1135</v>
       </c>
       <c r="E511" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="512" spans="1:5">
@@ -13233,7 +12915,7 @@
         <v>1136</v>
       </c>
       <c r="E512" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="513" spans="1:5">
@@ -13250,7 +12932,7 @@
         <v>1137</v>
       </c>
       <c r="E513" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="514" spans="1:5">
@@ -13267,7 +12949,7 @@
         <v>1138</v>
       </c>
       <c r="E514" t="s">
-        <v>1384</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="515" spans="1:5">
@@ -13284,7 +12966,7 @@
         <v>1139</v>
       </c>
       <c r="E515" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="516" spans="1:5">
@@ -13301,7 +12983,7 @@
         <v>1140</v>
       </c>
       <c r="E516" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="517" spans="1:5">
@@ -13318,7 +13000,7 @@
         <v>1141</v>
       </c>
       <c r="E517" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="518" spans="1:5">
@@ -13335,7 +13017,7 @@
         <v>1142</v>
       </c>
       <c r="E518" t="s">
-        <v>1384</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="519" spans="1:5">
@@ -13352,7 +13034,7 @@
         <v>1143</v>
       </c>
       <c r="E519" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="520" spans="1:5">
@@ -13369,7 +13051,7 @@
         <v>1144</v>
       </c>
       <c r="E520" t="s">
-        <v>1384</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="521" spans="1:5">
@@ -13386,7 +13068,7 @@
         <v>1145</v>
       </c>
       <c r="E521" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="522" spans="1:5">
@@ -13403,7 +13085,7 @@
         <v>1146</v>
       </c>
       <c r="E522" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="523" spans="1:5">
@@ -13420,7 +13102,7 @@
         <v>1147</v>
       </c>
       <c r="E523" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="524" spans="1:5">
@@ -13437,7 +13119,7 @@
         <v>1148</v>
       </c>
       <c r="E524" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="525" spans="1:5">
@@ -13454,7 +13136,7 @@
         <v>1149</v>
       </c>
       <c r="E525" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="526" spans="1:5">
@@ -13471,7 +13153,7 @@
         <v>1150</v>
       </c>
       <c r="E526" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="527" spans="1:5">
@@ -13488,7 +13170,7 @@
         <v>1151</v>
       </c>
       <c r="E527" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="528" spans="1:5">
@@ -13505,7 +13187,7 @@
         <v>1152</v>
       </c>
       <c r="E528" t="s">
-        <v>1384</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="529" spans="1:5">
@@ -13522,7 +13204,7 @@
         <v>1153</v>
       </c>
       <c r="E529" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="530" spans="1:5">
@@ -13539,7 +13221,7 @@
         <v>1154</v>
       </c>
       <c r="E530" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="531" spans="1:5">
@@ -13556,7 +13238,7 @@
         <v>1155</v>
       </c>
       <c r="E531" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="532" spans="1:5">
@@ -13573,7 +13255,7 @@
         <v>1156</v>
       </c>
       <c r="E532" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="533" spans="1:5">
@@ -13590,7 +13272,7 @@
         <v>1157</v>
       </c>
       <c r="E533" t="s">
-        <v>1384</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="534" spans="1:5">
@@ -13607,7 +13289,7 @@
         <v>1158</v>
       </c>
       <c r="E534" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="535" spans="1:5">
@@ -13624,7 +13306,7 @@
         <v>1159</v>
       </c>
       <c r="E535" t="s">
-        <v>1384</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="536" spans="1:5">
@@ -13641,7 +13323,7 @@
         <v>1160</v>
       </c>
       <c r="E536" t="s">
-        <v>1384</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="537" spans="1:5">
@@ -13658,7 +13340,7 @@
         <v>1161</v>
       </c>
       <c r="E537" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="538" spans="1:5">
@@ -13675,7 +13357,7 @@
         <v>1162</v>
       </c>
       <c r="E538" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="539" spans="1:5">
@@ -13692,7 +13374,7 @@
         <v>1163</v>
       </c>
       <c r="E539" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="540" spans="1:5">
@@ -13709,7 +13391,7 @@
         <v>1164</v>
       </c>
       <c r="E540" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="541" spans="1:5">
@@ -13726,7 +13408,7 @@
         <v>1165</v>
       </c>
       <c r="E541" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="542" spans="1:5">
@@ -13743,7 +13425,7 @@
         <v>1166</v>
       </c>
       <c r="E542" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="543" spans="1:5">
@@ -13760,7 +13442,7 @@
         <v>1167</v>
       </c>
       <c r="E543" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="544" spans="1:5">
@@ -13777,7 +13459,7 @@
         <v>1168</v>
       </c>
       <c r="E544" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="545" spans="1:5">
@@ -13794,7 +13476,7 @@
         <v>1169</v>
       </c>
       <c r="E545" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="546" spans="1:5">
@@ -13811,7 +13493,7 @@
         <v>1170</v>
       </c>
       <c r="E546" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="547" spans="1:5">
@@ -13828,7 +13510,7 @@
         <v>1171</v>
       </c>
       <c r="E547" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="548" spans="1:5">
@@ -13845,7 +13527,7 @@
         <v>1172</v>
       </c>
       <c r="E548" t="s">
-        <v>1384</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="549" spans="1:5">
@@ -13862,7 +13544,7 @@
         <v>1173</v>
       </c>
       <c r="E549" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="550" spans="1:5">
@@ -13879,7 +13561,7 @@
         <v>1174</v>
       </c>
       <c r="E550" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="551" spans="1:5">
@@ -13896,7 +13578,7 @@
         <v>1175</v>
       </c>
       <c r="E551" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="552" spans="1:5">
@@ -13913,7 +13595,7 @@
         <v>1176</v>
       </c>
       <c r="E552" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="553" spans="1:5">
@@ -13930,7 +13612,7 @@
         <v>1177</v>
       </c>
       <c r="E553" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="554" spans="1:5">
@@ -13947,7 +13629,7 @@
         <v>1178</v>
       </c>
       <c r="E554" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="555" spans="1:5">
@@ -13964,7 +13646,7 @@
         <v>1179</v>
       </c>
       <c r="E555" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="556" spans="1:5">
@@ -13981,7 +13663,7 @@
         <v>1180</v>
       </c>
       <c r="E556" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="557" spans="1:5">
@@ -13998,7 +13680,7 @@
         <v>1181</v>
       </c>
       <c r="E557" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="558" spans="1:5">
@@ -14015,7 +13697,7 @@
         <v>1182</v>
       </c>
       <c r="E558" t="s">
-        <v>1384</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="559" spans="1:5">
@@ -14032,7 +13714,7 @@
         <v>728</v>
       </c>
       <c r="E559" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="560" spans="1:5">
@@ -14049,7 +13731,7 @@
         <v>1183</v>
       </c>
       <c r="E560" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="561" spans="1:5">
@@ -14066,7 +13748,7 @@
         <v>1184</v>
       </c>
       <c r="E561" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="562" spans="1:5">
@@ -14083,7 +13765,7 @@
         <v>1185</v>
       </c>
       <c r="E562" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="563" spans="1:5">
@@ -14100,7 +13782,7 @@
         <v>1186</v>
       </c>
       <c r="E563" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="564" spans="1:5">
@@ -14117,7 +13799,7 @@
         <v>1187</v>
       </c>
       <c r="E564" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="565" spans="1:5">
@@ -14134,7 +13816,7 @@
         <v>1188</v>
       </c>
       <c r="E565" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="566" spans="1:5">
@@ -14151,7 +13833,7 @@
         <v>1189</v>
       </c>
       <c r="E566" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="567" spans="1:5">
@@ -14168,7 +13850,7 @@
         <v>1190</v>
       </c>
       <c r="E567" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="568" spans="1:5">
@@ -14185,7 +13867,7 @@
         <v>1191</v>
       </c>
       <c r="E568" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="569" spans="1:5">
@@ -14202,7 +13884,7 @@
         <v>1192</v>
       </c>
       <c r="E569" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="570" spans="1:5">
@@ -14219,7 +13901,7 @@
         <v>1193</v>
       </c>
       <c r="E570" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="571" spans="1:5">
@@ -14236,7 +13918,7 @@
         <v>1194</v>
       </c>
       <c r="E571" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="572" spans="1:5">
@@ -14253,7 +13935,7 @@
         <v>1195</v>
       </c>
       <c r="E572" t="s">
-        <v>1384</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="573" spans="1:5">
@@ -14270,7 +13952,7 @@
         <v>1196</v>
       </c>
       <c r="E573" t="s">
-        <v>1384</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="574" spans="1:5">
@@ -14287,7 +13969,7 @@
         <v>1197</v>
       </c>
       <c r="E574" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="575" spans="1:5">
@@ -14304,7 +13986,7 @@
         <v>1198</v>
       </c>
       <c r="E575" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="576" spans="1:5">
@@ -14321,7 +14003,7 @@
         <v>1199</v>
       </c>
       <c r="E576" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="577" spans="1:5">
@@ -14338,7 +14020,7 @@
         <v>1200</v>
       </c>
       <c r="E577" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="578" spans="1:5">
@@ -14355,7 +14037,7 @@
         <v>1201</v>
       </c>
       <c r="E578" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="579" spans="1:5">
@@ -14372,7 +14054,7 @@
         <v>1202</v>
       </c>
       <c r="E579" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="580" spans="1:5">
@@ -14389,7 +14071,7 @@
         <v>1203</v>
       </c>
       <c r="E580" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="581" spans="1:5">
@@ -14406,7 +14088,7 @@
         <v>1204</v>
       </c>
       <c r="E581" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="582" spans="1:5">
@@ -14423,7 +14105,7 @@
         <v>1205</v>
       </c>
       <c r="E582" t="s">
-        <v>1384</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="583" spans="1:5">
@@ -14440,7 +14122,7 @@
         <v>1206</v>
       </c>
       <c r="E583" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="584" spans="1:5">
@@ -14457,7 +14139,7 @@
         <v>1207</v>
       </c>
       <c r="E584" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="585" spans="1:5">
@@ -14474,7 +14156,7 @@
         <v>1208</v>
       </c>
       <c r="E585" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="586" spans="1:5">
@@ -14491,7 +14173,7 @@
         <v>1209</v>
       </c>
       <c r="E586" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="587" spans="1:5">
@@ -14508,7 +14190,7 @@
         <v>1210</v>
       </c>
       <c r="E587" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="588" spans="1:5">
@@ -14525,7 +14207,7 @@
         <v>1211</v>
       </c>
       <c r="E588" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="589" spans="1:5">
@@ -14542,7 +14224,7 @@
         <v>1212</v>
       </c>
       <c r="E589" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="590" spans="1:5">
@@ -14559,7 +14241,7 @@
         <v>1213</v>
       </c>
       <c r="E590" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="591" spans="1:5">
@@ -14576,7 +14258,7 @@
         <v>1214</v>
       </c>
       <c r="E591" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="592" spans="1:5">
@@ -14593,7 +14275,7 @@
         <v>1215</v>
       </c>
       <c r="E592" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="593" spans="1:5">
@@ -14610,7 +14292,7 @@
         <v>1216</v>
       </c>
       <c r="E593" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="594" spans="1:5">
@@ -14627,7 +14309,7 @@
         <v>1217</v>
       </c>
       <c r="E594" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="595" spans="1:5">
@@ -14644,7 +14326,7 @@
         <v>1218</v>
       </c>
       <c r="E595" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="596" spans="1:5">
@@ -14661,7 +14343,7 @@
         <v>1219</v>
       </c>
       <c r="E596" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="597" spans="1:5">
@@ -14678,7 +14360,7 @@
         <v>1220</v>
       </c>
       <c r="E597" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="598" spans="1:5">
@@ -14695,7 +14377,7 @@
         <v>1221</v>
       </c>
       <c r="E598" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="599" spans="1:5">
@@ -14712,7 +14394,7 @@
         <v>1222</v>
       </c>
       <c r="E599" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="600" spans="1:5">
@@ -14729,7 +14411,7 @@
         <v>1223</v>
       </c>
       <c r="E600" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="601" spans="1:5">
@@ -14746,7 +14428,7 @@
         <v>1224</v>
       </c>
       <c r="E601" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="602" spans="1:5">
@@ -14763,7 +14445,7 @@
         <v>1225</v>
       </c>
       <c r="E602" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="603" spans="1:5">
@@ -14780,7 +14462,7 @@
         <v>1226</v>
       </c>
       <c r="E603" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="604" spans="1:5">
@@ -14797,7 +14479,7 @@
         <v>1227</v>
       </c>
       <c r="E604" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="605" spans="1:5">
@@ -14814,7 +14496,7 @@
         <v>1228</v>
       </c>
       <c r="E605" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="606" spans="1:5">
@@ -14831,7 +14513,7 @@
         <v>1229</v>
       </c>
       <c r="E606" t="s">
-        <v>1384</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="607" spans="1:5">
@@ -14848,7 +14530,7 @@
         <v>1230</v>
       </c>
       <c r="E607" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="608" spans="1:5">
@@ -14865,7 +14547,7 @@
         <v>1231</v>
       </c>
       <c r="E608" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="609" spans="1:5">
@@ -14882,7 +14564,7 @@
         <v>1232</v>
       </c>
       <c r="E609" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="610" spans="1:5">
@@ -14899,7 +14581,7 @@
         <v>1233</v>
       </c>
       <c r="E610" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="611" spans="1:5">
@@ -14916,7 +14598,7 @@
         <v>1234</v>
       </c>
       <c r="E611" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="612" spans="1:5">
@@ -14933,7 +14615,7 @@
         <v>1235</v>
       </c>
       <c r="E612" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="613" spans="1:5">
@@ -14950,7 +14632,7 @@
         <v>1236</v>
       </c>
       <c r="E613" t="s">
-        <v>1384</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="614" spans="1:5">
@@ -14967,7 +14649,7 @@
         <v>1237</v>
       </c>
       <c r="E614" t="s">
-        <v>1384</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="615" spans="1:5">
@@ -14984,7 +14666,7 @@
         <v>1238</v>
       </c>
       <c r="E615" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="616" spans="1:5">
@@ -15001,7 +14683,7 @@
         <v>1239</v>
       </c>
       <c r="E616" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="617" spans="1:5">
@@ -15018,7 +14700,7 @@
         <v>1240</v>
       </c>
       <c r="E617" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="618" spans="1:5">
@@ -15035,7 +14717,7 @@
         <v>1241</v>
       </c>
       <c r="E618" t="s">
-        <v>1385</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="619" spans="1:5">
@@ -15052,7 +14734,7 @@
         <v>1242</v>
       </c>
       <c r="E619" t="s">
-        <v>1385</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="620" spans="1:5">
@@ -15069,7 +14751,7 @@
         <v>1243</v>
       </c>
       <c r="E620" t="s">
-        <v>1385</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="621" spans="1:5">
@@ -15086,7 +14768,7 @@
         <v>1244</v>
       </c>
       <c r="E621" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="622" spans="1:5">
@@ -15103,7 +14785,7 @@
         <v>1245</v>
       </c>
       <c r="E622" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="623" spans="1:5">
@@ -15120,7 +14802,7 @@
         <v>1246</v>
       </c>
       <c r="E623" t="s">
-        <v>1385</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="624" spans="1:5">
@@ -15137,7 +14819,7 @@
         <v>1247</v>
       </c>
       <c r="E624" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="625" spans="1:5">
@@ -15154,7 +14836,7 @@
         <v>1248</v>
       </c>
       <c r="E625" t="s">
-        <v>1385</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="626" spans="1:5">
@@ -15171,7 +14853,7 @@
         <v>1249</v>
       </c>
       <c r="E626" t="s">
-        <v>1385</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="627" spans="1:5">
@@ -15188,7 +14870,7 @@
         <v>1250</v>
       </c>
       <c r="E627" t="s">
-        <v>1385</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="628" spans="1:5">
@@ -15205,7 +14887,7 @@
         <v>1251</v>
       </c>
       <c r="E628" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="629" spans="1:5">
@@ -15222,7 +14904,7 @@
         <v>1252</v>
       </c>
       <c r="E629" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="630" spans="1:5">
@@ -15239,7 +14921,7 @@
         <v>1253</v>
       </c>
       <c r="E630" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="631" spans="1:5">
@@ -15256,7 +14938,7 @@
         <v>1254</v>
       </c>
       <c r="E631" t="s">
-        <v>1385</v>
+        <v>1255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>